<commit_message>
Updated feed to reflect fortnightly changes in animal feed management
</commit_message>
<xml_diff>
--- a/Tests/Validation/Stock/Keogh2023Observed.xlsx
+++ b/Tests/Validation/Stock/Keogh2023Observed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csiroau-my.sharepoint.com/personal/keo027_csiro_au/Documents/Documents/CSIRO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1621A78E-474D-4023-8AA2-AD66A6D31FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="8_{1621A78E-474D-4023-8AA2-AD66A6D31FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7B26189-195A-436A-8C22-8B0D59470CB9}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidationData" sheetId="1" r:id="rId1"/>
@@ -508,7 +508,7 @@
       </c>
       <c r="D2" s="1"/>
       <c r="F2" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G2" s="3">
         <v>32.299999999999997</v>
@@ -528,12 +528,12 @@
       </c>
       <c r="D3" s="1"/>
       <c r="F3" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3">
         <f>H2+F3/1000</f>
-        <v>1.3547696159444444</v>
+        <v>1.1429810648148149</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -550,12 +550,12 @@
       </c>
       <c r="D4" s="1"/>
       <c r="F4" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4">
         <f t="shared" ref="H4:H58" si="2">H3+F4/1000</f>
-        <v>2.7095392318888889</v>
+        <v>2.2859621296296297</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -572,12 +572,12 @@
       </c>
       <c r="D5" s="1"/>
       <c r="F5" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5">
         <f t="shared" si="2"/>
-        <v>4.0643088478333329</v>
+        <v>3.4289431944444448</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -594,12 +594,12 @@
       </c>
       <c r="D6" s="1"/>
       <c r="F6" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6">
         <f t="shared" si="2"/>
-        <v>5.4190784637777778</v>
+        <v>4.5719242592592595</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -616,12 +616,12 @@
       </c>
       <c r="D7" s="1"/>
       <c r="F7" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7">
         <f t="shared" si="2"/>
-        <v>6.7738480797222227</v>
+        <v>5.7149053240740741</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -638,12 +638,12 @@
       </c>
       <c r="D8" s="1"/>
       <c r="F8" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8">
         <f t="shared" si="2"/>
-        <v>8.1286176956666676</v>
+        <v>6.8578863888888888</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -660,12 +660,12 @@
       </c>
       <c r="D9" s="1"/>
       <c r="F9" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9">
         <f t="shared" si="2"/>
-        <v>9.4833873116111125</v>
+        <v>8.0008674537037034</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -682,12 +682,12 @@
       </c>
       <c r="D10" s="1"/>
       <c r="F10" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10">
         <f t="shared" si="2"/>
-        <v>10.838156927555557</v>
+        <v>9.143848518518519</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -704,12 +704,12 @@
       </c>
       <c r="D11" s="1"/>
       <c r="F11" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11">
         <f t="shared" si="2"/>
-        <v>12.192926543500002</v>
+        <v>10.286829583333335</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -726,12 +726,12 @@
       </c>
       <c r="D12" s="1"/>
       <c r="F12" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12">
         <f t="shared" si="2"/>
-        <v>13.547696159444447</v>
+        <v>11.42981064814815</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -748,12 +748,12 @@
       </c>
       <c r="D13" s="1"/>
       <c r="F13" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13">
         <f t="shared" si="2"/>
-        <v>14.902465775388892</v>
+        <v>12.572791712962966</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -770,12 +770,12 @@
       </c>
       <c r="D14" s="1"/>
       <c r="F14" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14">
         <f t="shared" si="2"/>
-        <v>16.257235391333335</v>
+        <v>13.715772777777781</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -792,12 +792,12 @@
       </c>
       <c r="D15" s="1"/>
       <c r="F15" s="6">
-        <v>1354.7696159444445</v>
+        <v>1142.9810648148148</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15">
         <f t="shared" si="2"/>
-        <v>17.61200500727778</v>
+        <v>14.858753842592597</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -814,12 +814,12 @@
       </c>
       <c r="D16" s="1"/>
       <c r="F16" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16">
         <f t="shared" si="2"/>
-        <v>18.966774623222225</v>
+        <v>16.221228830246918</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -836,12 +836,12 @@
       </c>
       <c r="D17" s="1"/>
       <c r="F17" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17">
         <f t="shared" si="2"/>
-        <v>20.32154423916667</v>
+        <v>17.583703817901238</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -858,12 +858,12 @@
       </c>
       <c r="D18" s="1"/>
       <c r="F18" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18">
         <f t="shared" si="2"/>
-        <v>21.676313855111115</v>
+        <v>18.946178805555558</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -880,12 +880,12 @@
       </c>
       <c r="D19" s="1"/>
       <c r="F19" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19">
         <f t="shared" si="2"/>
-        <v>23.03108347105556</v>
+        <v>20.308653793209878</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
@@ -902,12 +902,12 @@
       </c>
       <c r="D20" s="1"/>
       <c r="F20" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20">
         <f t="shared" si="2"/>
-        <v>24.385853087000005</v>
+        <v>21.671128780864198</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -924,12 +924,12 @@
       </c>
       <c r="D21" s="1"/>
       <c r="F21" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21">
         <f t="shared" si="2"/>
-        <v>25.740622702944449</v>
+        <v>23.033603768518518</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -946,12 +946,12 @@
       </c>
       <c r="D22" s="1"/>
       <c r="F22" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22">
         <f t="shared" si="2"/>
-        <v>27.095392318888894</v>
+        <v>24.396078756172837</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
@@ -968,12 +968,12 @@
       </c>
       <c r="D23" s="1"/>
       <c r="F23" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23">
         <f t="shared" si="2"/>
-        <v>28.450161934833339</v>
+        <v>25.758553743827157</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
@@ -990,12 +990,12 @@
       </c>
       <c r="D24" s="1"/>
       <c r="F24" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24">
         <f t="shared" si="2"/>
-        <v>29.804931550777784</v>
+        <v>27.121028731481477</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
@@ -1012,12 +1012,12 @@
       </c>
       <c r="D25" s="1"/>
       <c r="F25" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25">
         <f t="shared" si="2"/>
-        <v>31.159701166722229</v>
+        <v>28.483503719135797</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
@@ -1034,12 +1034,12 @@
       </c>
       <c r="D26" s="1"/>
       <c r="F26" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26">
         <f t="shared" si="2"/>
-        <v>32.51447078266667</v>
+        <v>29.845978706790117</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -1056,12 +1056,12 @@
       </c>
       <c r="D27" s="1"/>
       <c r="F27" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27">
         <f t="shared" si="2"/>
-        <v>33.869240398611112</v>
+        <v>31.208453694444437</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -1078,12 +1078,12 @@
       </c>
       <c r="D28" s="1"/>
       <c r="F28" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28">
         <f t="shared" si="2"/>
-        <v>35.224010014555553</v>
+        <v>32.57092868209876</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
@@ -1100,12 +1100,12 @@
       </c>
       <c r="D29" s="1"/>
       <c r="F29" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29">
         <f t="shared" si="2"/>
-        <v>36.578779630499994</v>
+        <v>33.933403669753083</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D30" s="1"/>
       <c r="F30" s="6">
-        <v>1354.7696159444445</v>
+        <v>1362.4749876543208</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30">
         <f t="shared" si="2"/>
-        <v>37.933549246444436</v>
+        <v>35.295878657407407</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
@@ -1144,12 +1144,12 @@
       </c>
       <c r="D31" s="1"/>
       <c r="F31" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31">
         <f t="shared" si="2"/>
-        <v>39.288318862388877</v>
+        <v>36.72726633831909</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
@@ -1166,12 +1166,12 @@
       </c>
       <c r="D32" s="1"/>
       <c r="F32" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G32" s="3"/>
       <c r="H32">
         <f t="shared" si="2"/>
-        <v>40.643088478333318</v>
+        <v>38.158654019230774</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
@@ -1188,12 +1188,12 @@
       </c>
       <c r="D33" s="1"/>
       <c r="F33" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33">
         <f t="shared" si="2"/>
-        <v>41.99785809427776</v>
+        <v>39.590041700142457</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
@@ -1210,12 +1210,12 @@
       </c>
       <c r="D34" s="1"/>
       <c r="F34" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34">
         <f t="shared" si="2"/>
-        <v>43.352627710222201</v>
+        <v>41.021429381054141</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
@@ -1232,12 +1232,12 @@
       </c>
       <c r="D35" s="1"/>
       <c r="F35" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35">
         <f t="shared" si="2"/>
-        <v>44.707397326166642</v>
+        <v>42.452817061965824</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="D36" s="1"/>
       <c r="F36" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G36" s="3"/>
       <c r="H36">
         <f t="shared" si="2"/>
-        <v>46.062166942111084</v>
+        <v>43.884204742877507</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
@@ -1276,12 +1276,12 @@
       </c>
       <c r="D37" s="1"/>
       <c r="F37" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G37" s="3"/>
       <c r="H37">
         <f t="shared" si="2"/>
-        <v>47.416936558055525</v>
+        <v>45.315592423789191</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D38" s="1"/>
       <c r="F38" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G38" s="3"/>
       <c r="H38">
         <f t="shared" si="2"/>
-        <v>48.771706173999966</v>
+        <v>46.746980104700874</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
@@ -1320,12 +1320,12 @@
       </c>
       <c r="D39" s="1"/>
       <c r="F39" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39">
         <f t="shared" si="2"/>
-        <v>50.126475789944408</v>
+        <v>48.178367785612558</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="D40" s="1"/>
       <c r="F40" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40">
         <f t="shared" si="2"/>
-        <v>51.481245405888849</v>
+        <v>49.609755466524241</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
@@ -1364,12 +1364,12 @@
       </c>
       <c r="D41" s="1"/>
       <c r="F41" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G41" s="4"/>
       <c r="H41">
         <f t="shared" si="2"/>
-        <v>52.83601502183329</v>
+        <v>51.041143147435925</v>
       </c>
       <c r="I41" s="2"/>
     </row>
@@ -1387,12 +1387,12 @@
       </c>
       <c r="D42" s="1"/>
       <c r="F42" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G42" s="3"/>
       <c r="H42">
         <f t="shared" si="2"/>
-        <v>54.190784637777732</v>
+        <v>52.472530828347608</v>
       </c>
       <c r="I42" s="2"/>
     </row>
@@ -1410,12 +1410,12 @@
       </c>
       <c r="D43" s="1"/>
       <c r="F43" s="6">
-        <v>1354.7696159444445</v>
+        <v>1431.3876809116807</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43">
         <f t="shared" si="2"/>
-        <v>55.545554253722173</v>
+        <v>53.903918509259292</v>
       </c>
       <c r="I43" s="2"/>
     </row>
@@ -1433,12 +1433,12 @@
       </c>
       <c r="D44" s="1"/>
       <c r="F44" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44">
         <f t="shared" si="2"/>
-        <v>56.900323869666614</v>
+        <v>55.388724351851884</v>
       </c>
       <c r="I44" s="2"/>
     </row>
@@ -1456,12 +1456,12 @@
       </c>
       <c r="D45" s="1"/>
       <c r="F45" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G45" s="3"/>
       <c r="H45">
         <f t="shared" si="2"/>
-        <v>58.255093485611056</v>
+        <v>56.873530194444477</v>
       </c>
       <c r="I45" s="2"/>
     </row>
@@ -1479,12 +1479,12 @@
       </c>
       <c r="D46" s="1"/>
       <c r="F46" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46">
         <f t="shared" si="2"/>
-        <v>59.609863101555497</v>
+        <v>58.35833603703707</v>
       </c>
       <c r="I46" s="2"/>
     </row>
@@ -1502,12 +1502,12 @@
       </c>
       <c r="D47" s="1"/>
       <c r="F47" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G47" s="3"/>
       <c r="H47">
         <f t="shared" si="2"/>
-        <v>60.964632717499939</v>
+        <v>59.843141879629663</v>
       </c>
       <c r="I47" s="2"/>
     </row>
@@ -1525,12 +1525,12 @@
       </c>
       <c r="D48" s="1"/>
       <c r="F48" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G48" s="4"/>
       <c r="H48">
         <f t="shared" si="2"/>
-        <v>62.31940233344438</v>
+        <v>61.327947722222255</v>
       </c>
       <c r="I48" s="2"/>
     </row>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="D49" s="1"/>
       <c r="F49" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G49" s="4"/>
       <c r="H49">
         <f>H48+F49/1000</f>
-        <v>63.674171949388821</v>
+        <v>62.812753564814848</v>
       </c>
       <c r="I49" s="2"/>
     </row>
@@ -1571,12 +1571,12 @@
       </c>
       <c r="D50" s="1"/>
       <c r="F50" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G50" s="4"/>
       <c r="H50">
         <f t="shared" si="2"/>
-        <v>65.02894156533327</v>
+        <v>64.297559407407434</v>
       </c>
       <c r="I50" s="2"/>
     </row>
@@ -1594,12 +1594,12 @@
       </c>
       <c r="D51" s="1"/>
       <c r="F51" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G51" s="4"/>
       <c r="H51">
         <f t="shared" si="2"/>
-        <v>66.383711181277718</v>
+        <v>65.782365250000026</v>
       </c>
       <c r="I51" s="2"/>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="D52" s="1"/>
       <c r="F52" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G52" s="4"/>
       <c r="H52">
         <f t="shared" si="2"/>
-        <v>67.738480797222167</v>
+        <v>67.267171092592619</v>
       </c>
       <c r="I52" s="2"/>
     </row>
@@ -1640,12 +1640,12 @@
       </c>
       <c r="D53" s="1"/>
       <c r="F53" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G53" s="4"/>
       <c r="H53">
         <f t="shared" si="2"/>
-        <v>69.093250413166615</v>
+        <v>68.751976935185212</v>
       </c>
       <c r="I53" s="2"/>
     </row>
@@ -1663,12 +1663,12 @@
       </c>
       <c r="D54" s="1"/>
       <c r="F54" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G54" s="4"/>
       <c r="H54">
         <f t="shared" si="2"/>
-        <v>70.448020029111063</v>
+        <v>70.236782777777805</v>
       </c>
       <c r="I54" s="2"/>
     </row>
@@ -1686,12 +1686,12 @@
       </c>
       <c r="D55" s="1"/>
       <c r="F55" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G55" s="4"/>
       <c r="H55">
         <f t="shared" si="2"/>
-        <v>71.802789645055512</v>
+        <v>71.721588620370397</v>
       </c>
       <c r="I55" s="2"/>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="D56" s="1"/>
       <c r="F56" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G56" s="4"/>
       <c r="H56">
         <f t="shared" si="2"/>
-        <v>73.15755926099996</v>
+        <v>73.20639446296299</v>
       </c>
       <c r="I56" s="2"/>
     </row>
@@ -1732,12 +1732,12 @@
       </c>
       <c r="D57" s="1"/>
       <c r="F57" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G57" s="4"/>
       <c r="H57">
         <f t="shared" si="2"/>
-        <v>74.512328876944409</v>
+        <v>74.691200305555583</v>
       </c>
       <c r="I57" s="2"/>
     </row>
@@ -1755,14 +1755,14 @@
       </c>
       <c r="D58" s="1"/>
       <c r="F58" s="6">
-        <v>1354.7696159444445</v>
+        <v>1484.8058425925924</v>
       </c>
       <c r="G58" s="4">
         <v>44.4</v>
       </c>
       <c r="H58">
         <f t="shared" si="2"/>
-        <v>75.867098492888857</v>
+        <v>76.176006148148176</v>
       </c>
       <c r="I58" s="2"/>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D59" s="1"/>
       <c r="F59" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G59" s="4">
         <v>31.2</v>
@@ -1798,12 +1798,12 @@
         <v>19</v>
       </c>
       <c r="F60" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G60" s="3"/>
       <c r="H60">
         <f t="shared" ref="H60:H62" si="3">H59+F60/1000</f>
-        <v>0.84338389741509456</v>
+        <v>0.7997702546296297</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
@@ -1819,12 +1819,12 @@
         <v>19</v>
       </c>
       <c r="F61" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G61" s="3"/>
       <c r="H61">
         <f t="shared" si="3"/>
-        <v>1.6867677948301891</v>
+        <v>1.5995405092592594</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
@@ -1840,12 +1840,12 @@
         <v>19</v>
       </c>
       <c r="F62" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G62" s="3"/>
       <c r="H62">
         <f t="shared" si="3"/>
-        <v>2.5301516922452838</v>
+        <v>2.3993107638888889</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
@@ -1861,12 +1861,12 @@
         <v>19</v>
       </c>
       <c r="F63" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G63" s="4"/>
       <c r="H63">
         <f t="shared" ref="H63:H115" si="4">H62+F63/1000</f>
-        <v>3.3735355896603783</v>
+        <v>3.1990810185185188</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
@@ -1882,12 +1882,12 @@
         <v>19</v>
       </c>
       <c r="F64" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G64" s="3"/>
       <c r="H64">
         <f t="shared" si="4"/>
-        <v>4.2169194870754731</v>
+        <v>3.9988512731481487</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
@@ -1903,12 +1903,12 @@
         <v>19</v>
       </c>
       <c r="F65" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G65" s="3"/>
       <c r="H65">
         <f t="shared" si="4"/>
-        <v>5.0603033844905676</v>
+        <v>4.7986215277777786</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
@@ -1924,12 +1924,12 @@
         <v>19</v>
       </c>
       <c r="F66" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G66" s="3"/>
       <c r="H66">
         <f t="shared" si="4"/>
-        <v>5.9036872819056621</v>
+        <v>5.5983917824074085</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
@@ -1945,12 +1945,12 @@
         <v>19</v>
       </c>
       <c r="F67" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G67" s="3"/>
       <c r="H67">
         <f t="shared" si="4"/>
-        <v>6.7470711793207565</v>
+        <v>6.3981620370370385</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
@@ -1966,12 +1966,12 @@
         <v>19</v>
       </c>
       <c r="F68" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G68" s="3"/>
       <c r="H68">
         <f t="shared" si="4"/>
-        <v>7.590455076735851</v>
+        <v>7.1979322916666684</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
@@ -1987,12 +1987,12 @@
         <v>19</v>
       </c>
       <c r="F69" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G69" s="3"/>
       <c r="H69">
         <f t="shared" si="4"/>
-        <v>8.4338389741509463</v>
+        <v>7.9977025462962983</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
@@ -2008,12 +2008,12 @@
         <v>19</v>
       </c>
       <c r="F70" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G70" s="4"/>
       <c r="H70">
         <f t="shared" si="4"/>
-        <v>9.2772228715660408</v>
+        <v>8.7974728009259273</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
@@ -2029,12 +2029,12 @@
         <v>19</v>
       </c>
       <c r="F71" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G71" s="3"/>
       <c r="H71">
         <f t="shared" si="4"/>
-        <v>10.120606768981135</v>
+        <v>9.5972430555555572</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
@@ -2050,12 +2050,12 @@
         <v>19</v>
       </c>
       <c r="F72" s="6">
-        <v>843.38389741509457</v>
+        <v>799.77025462962968</v>
       </c>
       <c r="G72" s="3"/>
       <c r="H72">
         <f t="shared" si="4"/>
-        <v>10.96399066639623</v>
+        <v>10.397013310185187</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
@@ -2071,12 +2071,12 @@
         <v>19</v>
       </c>
       <c r="F73" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G73" s="3"/>
       <c r="H73">
         <f t="shared" si="4"/>
-        <v>11.807374563811324</v>
+        <v>11.234913310185187</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
@@ -2092,12 +2092,12 @@
         <v>19</v>
       </c>
       <c r="F74" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G74" s="3"/>
       <c r="H74">
         <f t="shared" si="4"/>
-        <v>12.650758461226419</v>
+        <v>12.072813310185186</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
@@ -2113,12 +2113,12 @@
         <v>19</v>
       </c>
       <c r="F75" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G75" s="3"/>
       <c r="H75">
         <f t="shared" si="4"/>
-        <v>13.494142358641513</v>
+        <v>12.910713310185185</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
@@ -2134,12 +2134,12 @@
         <v>19</v>
       </c>
       <c r="F76" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G76" s="3"/>
       <c r="H76">
         <f t="shared" si="4"/>
-        <v>14.337526256056607</v>
+        <v>13.748613310185185</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
@@ -2155,12 +2155,12 @@
         <v>19</v>
       </c>
       <c r="F77" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G77" s="4"/>
       <c r="H77">
         <f t="shared" si="4"/>
-        <v>15.180910153471702</v>
+        <v>14.586513310185184</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
@@ -2176,12 +2176,12 @@
         <v>19</v>
       </c>
       <c r="F78" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G78" s="3"/>
       <c r="H78">
         <f t="shared" si="4"/>
-        <v>16.024294050886798</v>
+        <v>15.424413310185184</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
@@ -2197,12 +2197,12 @@
         <v>19</v>
       </c>
       <c r="F79" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G79" s="3"/>
       <c r="H79">
         <f t="shared" si="4"/>
-        <v>16.867677948301893</v>
+        <v>16.262313310185185</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
@@ -2218,12 +2218,12 @@
         <v>19</v>
       </c>
       <c r="F80" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G80" s="3"/>
       <c r="H80">
         <f t="shared" si="4"/>
-        <v>17.711061845716987</v>
+        <v>17.100213310185186</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
@@ -2239,12 +2239,12 @@
         <v>19</v>
       </c>
       <c r="F81" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G81" s="3"/>
       <c r="H81">
         <f t="shared" si="4"/>
-        <v>18.554445743132082</v>
+        <v>17.938113310185187</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
@@ -2260,12 +2260,12 @@
         <v>19</v>
       </c>
       <c r="F82" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G82" s="3"/>
       <c r="H82">
         <f t="shared" si="4"/>
-        <v>19.397829640547176</v>
+        <v>18.776013310185188</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
@@ -2281,12 +2281,12 @@
         <v>19</v>
       </c>
       <c r="F83" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G83" s="3"/>
       <c r="H83">
         <f t="shared" si="4"/>
-        <v>20.24121353796227</v>
+        <v>19.61391331018519</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
@@ -2302,12 +2302,12 @@
         <v>19</v>
       </c>
       <c r="F84" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G84" s="4"/>
       <c r="H84">
         <f t="shared" si="4"/>
-        <v>21.084597435377365</v>
+        <v>20.451813310185191</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
@@ -2323,12 +2323,12 @@
         <v>19</v>
       </c>
       <c r="F85" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G85" s="3"/>
       <c r="H85">
         <f t="shared" si="4"/>
-        <v>21.927981332792459</v>
+        <v>21.289713310185192</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
@@ -2344,12 +2344,12 @@
         <v>19</v>
       </c>
       <c r="F86" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G86" s="3"/>
       <c r="H86">
         <f t="shared" si="4"/>
-        <v>22.771365230207554</v>
+        <v>22.127613310185193</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
@@ -2365,12 +2365,12 @@
         <v>19</v>
       </c>
       <c r="F87" s="6">
-        <v>843.38389741509457</v>
+        <v>837.89999999999975</v>
       </c>
       <c r="G87" s="3"/>
       <c r="H87">
         <f t="shared" si="4"/>
-        <v>23.614749127622648</v>
+        <v>22.965513310185194</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.3">
@@ -2386,12 +2386,12 @@
         <v>19</v>
       </c>
       <c r="F88" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G88" s="3"/>
       <c r="H88">
         <f t="shared" si="4"/>
-        <v>24.458133025037743</v>
+        <v>23.834136310185194</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
@@ -2407,12 +2407,12 @@
         <v>19</v>
       </c>
       <c r="F89" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G89" s="3"/>
       <c r="H89">
         <f t="shared" si="4"/>
-        <v>25.301516922452837</v>
+        <v>24.702759310185193</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.3">
@@ -2428,12 +2428,12 @@
         <v>19</v>
       </c>
       <c r="F90" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G90" s="3"/>
       <c r="H90">
         <f t="shared" si="4"/>
-        <v>26.144900819867932</v>
+        <v>25.571382310185193</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.3">
@@ -2449,12 +2449,12 @@
         <v>19</v>
       </c>
       <c r="F91" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G91" s="4"/>
       <c r="H91">
         <f t="shared" si="4"/>
-        <v>26.988284717283026</v>
+        <v>26.440005310185192</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.3">
@@ -2470,12 +2470,12 @@
         <v>19</v>
       </c>
       <c r="F92" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G92" s="3"/>
       <c r="H92">
         <f t="shared" si="4"/>
-        <v>27.83166861469812</v>
+        <v>27.308628310185192</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.3">
@@ -2491,12 +2491,12 @@
         <v>19</v>
       </c>
       <c r="F93" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G93" s="3"/>
       <c r="H93">
         <f t="shared" si="4"/>
-        <v>28.675052512113215</v>
+        <v>28.177251310185191</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.3">
@@ -2512,12 +2512,12 @@
         <v>19</v>
       </c>
       <c r="F94" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G94" s="3"/>
       <c r="H94">
         <f t="shared" si="4"/>
-        <v>29.518436409528309</v>
+        <v>29.045874310185191</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.3">
@@ -2533,12 +2533,12 @@
         <v>19</v>
       </c>
       <c r="F95" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G95" s="3"/>
       <c r="H95">
         <f t="shared" si="4"/>
-        <v>30.361820306943404</v>
+        <v>29.91449731018519</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.3">
@@ -2554,12 +2554,12 @@
         <v>19</v>
       </c>
       <c r="F96" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G96" s="3"/>
       <c r="H96">
         <f t="shared" si="4"/>
-        <v>31.205204204358498</v>
+        <v>30.78312031018519</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
@@ -2575,12 +2575,12 @@
         <v>19</v>
       </c>
       <c r="F97" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G97" s="3"/>
       <c r="H97">
         <f t="shared" si="4"/>
-        <v>32.048588101773596</v>
+        <v>31.651743310185189</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
@@ -2596,12 +2596,12 @@
         <v>19</v>
       </c>
       <c r="F98" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G98" s="4"/>
       <c r="H98">
         <f t="shared" si="4"/>
-        <v>32.891971999188691</v>
+        <v>32.520366310185189</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.3">
@@ -2617,12 +2617,12 @@
         <v>19</v>
       </c>
       <c r="F99" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G99" s="3"/>
       <c r="H99">
         <f t="shared" si="4"/>
-        <v>33.735355896603785</v>
+        <v>33.388989310185188</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.3">
@@ -2638,12 +2638,12 @@
         <v>19</v>
       </c>
       <c r="F100" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G100" s="3"/>
       <c r="H100">
         <f t="shared" si="4"/>
-        <v>34.57873979401888</v>
+        <v>34.257612310185188</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
@@ -2659,12 +2659,12 @@
         <v>19</v>
       </c>
       <c r="F101" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G101" s="3"/>
       <c r="H101">
         <f t="shared" si="4"/>
-        <v>35.422123691433974</v>
+        <v>35.126235310185187</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.3">
@@ -2680,12 +2680,12 @@
         <v>19</v>
       </c>
       <c r="F102" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G102" s="3"/>
       <c r="H102">
         <f t="shared" si="4"/>
-        <v>36.265507588849069</v>
+        <v>35.994858310185187</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
@@ -2701,12 +2701,12 @@
         <v>19</v>
       </c>
       <c r="F103" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G103" s="3"/>
       <c r="H103">
         <f t="shared" si="4"/>
-        <v>37.108891486264163</v>
+        <v>36.863481310185186</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.3">
@@ -2722,12 +2722,12 @@
         <v>19</v>
       </c>
       <c r="F104" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G104" s="3"/>
       <c r="H104">
         <f t="shared" si="4"/>
-        <v>37.952275383679257</v>
+        <v>37.732104310185186</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.3">
@@ -2743,12 +2743,12 @@
         <v>19</v>
       </c>
       <c r="F105" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G105" s="4"/>
       <c r="H105">
         <f t="shared" si="4"/>
-        <v>38.795659281094352</v>
+        <v>38.600727310185185</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.3">
@@ -2764,12 +2764,12 @@
         <v>19</v>
       </c>
       <c r="F106" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G106" s="4"/>
       <c r="H106">
         <f t="shared" si="4"/>
-        <v>39.639043178509446</v>
+        <v>39.469350310185185</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.3">
@@ -2785,12 +2785,12 @@
         <v>19</v>
       </c>
       <c r="F107" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G107" s="4"/>
       <c r="H107">
         <f t="shared" si="4"/>
-        <v>40.482427075924541</v>
+        <v>40.337973310185184</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.3">
@@ -2806,12 +2806,12 @@
         <v>19</v>
       </c>
       <c r="F108" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G108" s="4"/>
       <c r="H108">
         <f t="shared" si="4"/>
-        <v>41.325810973339635</v>
+        <v>41.206596310185184</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.3">
@@ -2827,12 +2827,12 @@
         <v>19</v>
       </c>
       <c r="F109" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G109" s="4"/>
       <c r="H109">
         <f t="shared" si="4"/>
-        <v>42.16919487075473</v>
+        <v>42.075219310185183</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.3">
@@ -2848,12 +2848,12 @@
         <v>19</v>
       </c>
       <c r="F110" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G110" s="4"/>
       <c r="H110">
         <f t="shared" si="4"/>
-        <v>43.012578768169824</v>
+        <v>42.943842310185182</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.3">
@@ -2869,12 +2869,12 @@
         <v>19</v>
       </c>
       <c r="F111" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G111" s="4"/>
       <c r="H111">
         <f t="shared" si="4"/>
-        <v>43.855962665584919</v>
+        <v>43.812465310185182</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.3">
@@ -2890,12 +2890,12 @@
         <v>19</v>
       </c>
       <c r="F112" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G112" s="4"/>
       <c r="H112">
         <f t="shared" si="4"/>
-        <v>44.699346563000013</v>
+        <v>44.681088310185181</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.3">
@@ -2911,12 +2911,12 @@
         <v>19</v>
       </c>
       <c r="F113" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G113" s="4"/>
       <c r="H113">
         <f t="shared" si="4"/>
-        <v>45.542730460415108</v>
+        <v>45.549711310185181</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.3">
@@ -2932,12 +2932,12 @@
         <v>19</v>
       </c>
       <c r="F114" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G114" s="4"/>
       <c r="H114">
         <f t="shared" si="4"/>
-        <v>46.386114357830202</v>
+        <v>46.41833431018518</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.3">
@@ -2953,14 +2953,14 @@
         <v>19</v>
       </c>
       <c r="F115" s="6">
-        <v>843.38389741509457</v>
+        <v>868.62299999999971</v>
       </c>
       <c r="G115" s="4">
         <v>36</v>
       </c>
       <c r="H115">
         <f t="shared" si="4"/>
-        <v>47.229498255245296</v>
+        <v>47.28695731018518</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.3">
@@ -2975,7 +2975,7 @@
         <v>20</v>
       </c>
       <c r="F116" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G116" s="4">
         <v>40.5</v>
@@ -2994,12 +2994,12 @@
         <v>20</v>
       </c>
       <c r="F117" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G117" s="3"/>
       <c r="H117">
         <f t="shared" ref="H116:H119" si="7">H116+F117/1000</f>
-        <v>1.4918147085555558</v>
+        <v>1.185390642857143</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.3">
@@ -3015,12 +3015,12 @@
         <v>20</v>
       </c>
       <c r="F118" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G118" s="3"/>
       <c r="H118">
         <f t="shared" si="7"/>
-        <v>2.9836294171111115</v>
+        <v>2.370781285714286</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.3">
@@ -3036,12 +3036,12 @@
         <v>20</v>
       </c>
       <c r="F119" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G119" s="3"/>
       <c r="H119">
         <f t="shared" si="7"/>
-        <v>4.4754441256666677</v>
+        <v>3.5561719285714291</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.3">
@@ -3057,12 +3057,12 @@
         <v>20</v>
       </c>
       <c r="F120" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G120" s="4"/>
       <c r="H120">
         <f t="shared" ref="H120:H182" si="8">H119+F120/1000</f>
-        <v>5.967258834222223</v>
+        <v>4.7415625714285721</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.3">
@@ -3078,12 +3078,12 @@
         <v>20</v>
       </c>
       <c r="F121" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G121" s="3"/>
       <c r="H121">
         <f t="shared" si="8"/>
-        <v>7.4590735427777783</v>
+        <v>5.9269532142857155</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.3">
@@ -3099,12 +3099,12 @@
         <v>20</v>
       </c>
       <c r="F122" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G122" s="3"/>
       <c r="H122">
         <f t="shared" si="8"/>
-        <v>8.9508882513333337</v>
+        <v>7.112343857142859</v>
       </c>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.3">
@@ -3120,12 +3120,12 @@
         <v>20</v>
       </c>
       <c r="F123" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G123" s="3"/>
       <c r="H123">
         <f t="shared" si="8"/>
-        <v>10.442702959888889</v>
+        <v>8.2977345000000025</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.3">
@@ -3141,12 +3141,12 @@
         <v>20</v>
       </c>
       <c r="F124" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G124" s="3"/>
       <c r="H124">
         <f t="shared" si="8"/>
-        <v>11.934517668444444</v>
+        <v>9.4831251428571459</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.3">
@@ -3162,12 +3162,12 @@
         <v>20</v>
       </c>
       <c r="F125" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G125" s="3"/>
       <c r="H125">
         <f t="shared" si="8"/>
-        <v>13.426332377</v>
+        <v>10.668515785714289</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.3">
@@ -3183,12 +3183,12 @@
         <v>20</v>
       </c>
       <c r="F126" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G126" s="3"/>
       <c r="H126">
         <f t="shared" si="8"/>
-        <v>14.918147085555555</v>
+        <v>11.853906428571433</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.3">
@@ -3204,12 +3204,12 @@
         <v>20</v>
       </c>
       <c r="F127" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G127" s="4"/>
       <c r="H127">
         <f t="shared" si="8"/>
-        <v>16.409961794111112</v>
+        <v>13.039297071428576</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.3">
@@ -3225,12 +3225,12 @@
         <v>20</v>
       </c>
       <c r="F128" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G128" s="3"/>
       <c r="H128">
         <f t="shared" si="8"/>
-        <v>17.901776502666667</v>
+        <v>14.22468771428572</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.3">
@@ -3246,12 +3246,12 @@
         <v>20</v>
       </c>
       <c r="F129" s="6">
-        <v>1491.8147085555559</v>
+        <v>1185.3906428571431</v>
       </c>
       <c r="G129" s="3"/>
       <c r="H129">
         <f t="shared" si="8"/>
-        <v>19.393591211222223</v>
+        <v>15.410078357142863</v>
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.3">
@@ -3267,12 +3267,12 @@
         <v>20</v>
       </c>
       <c r="F130" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G130" s="3"/>
       <c r="H130">
         <f t="shared" si="8"/>
-        <v>20.885405919777778</v>
+        <v>16.791555066666671</v>
       </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.3">
@@ -3288,12 +3288,12 @@
         <v>20</v>
       </c>
       <c r="F131" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G131" s="3"/>
       <c r="H131">
         <f t="shared" si="8"/>
-        <v>22.377220628333333</v>
+        <v>18.173031776190481</v>
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.3">
@@ -3309,12 +3309,12 @@
         <v>20</v>
       </c>
       <c r="F132" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G132" s="3"/>
       <c r="H132">
         <f t="shared" si="8"/>
-        <v>23.869035336888889</v>
+        <v>19.55450848571429</v>
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.3">
@@ -3330,12 +3330,12 @@
         <v>20</v>
       </c>
       <c r="F133" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G133" s="3"/>
       <c r="H133">
         <f t="shared" si="8"/>
-        <v>25.360850045444444</v>
+        <v>20.9359851952381</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.3">
@@ -3351,12 +3351,12 @@
         <v>20</v>
       </c>
       <c r="F134" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G134" s="4"/>
       <c r="H134">
         <f t="shared" si="8"/>
-        <v>26.852664753999999</v>
+        <v>22.31746190476191</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.3">
@@ -3372,12 +3372,12 @@
         <v>20</v>
       </c>
       <c r="F135" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G135" s="3"/>
       <c r="H135">
         <f t="shared" si="8"/>
-        <v>28.344479462555555</v>
+        <v>23.698938614285719</v>
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.3">
@@ -3393,12 +3393,12 @@
         <v>20</v>
       </c>
       <c r="F136" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G136" s="3"/>
       <c r="H136">
         <f t="shared" si="8"/>
-        <v>29.83629417111111</v>
+        <v>25.080415323809529</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.3">
@@ -3414,12 +3414,12 @@
         <v>20</v>
       </c>
       <c r="F137" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G137" s="3"/>
       <c r="H137">
         <f t="shared" si="8"/>
-        <v>31.328108879666665</v>
+        <v>26.461892033333339</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.3">
@@ -3435,12 +3435,12 @@
         <v>20</v>
       </c>
       <c r="F138" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G138" s="3"/>
       <c r="H138">
         <f t="shared" si="8"/>
-        <v>32.819923588222224</v>
+        <v>27.843368742857148</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.3">
@@ -3456,12 +3456,12 @@
         <v>20</v>
       </c>
       <c r="F139" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G139" s="3"/>
       <c r="H139">
         <f t="shared" si="8"/>
-        <v>34.311738296777783</v>
+        <v>29.224845452380958</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.3">
@@ -3477,12 +3477,12 @@
         <v>20</v>
       </c>
       <c r="F140" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G140" s="3"/>
       <c r="H140">
         <f t="shared" si="8"/>
-        <v>35.803553005333342</v>
+        <v>30.606322161904767</v>
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.3">
@@ -3498,12 +3498,12 @@
         <v>20</v>
       </c>
       <c r="F141" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G141" s="4"/>
       <c r="H141">
         <f t="shared" si="8"/>
-        <v>37.295367713888901</v>
+        <v>31.987798871428577</v>
       </c>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.3">
@@ -3519,12 +3519,12 @@
         <v>20</v>
       </c>
       <c r="F142" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G142" s="3"/>
       <c r="H142">
         <f t="shared" si="8"/>
-        <v>38.787182422444459</v>
+        <v>33.369275580952383</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.3">
@@ -3540,12 +3540,12 @@
         <v>20</v>
       </c>
       <c r="F143" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G143" s="3"/>
       <c r="H143">
         <f t="shared" si="8"/>
-        <v>40.278997131000018</v>
+        <v>34.750752290476193</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.3">
@@ -3561,12 +3561,12 @@
         <v>20</v>
       </c>
       <c r="F144" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238094</v>
       </c>
       <c r="G144" s="3"/>
       <c r="H144">
         <f t="shared" si="8"/>
-        <v>41.770811839555577</v>
+        <v>36.132229000000002</v>
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.3">
@@ -3582,12 +3582,12 @@
         <v>20</v>
       </c>
       <c r="F145" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G145" s="3"/>
       <c r="H145">
         <f t="shared" si="8"/>
-        <v>43.262626548111136</v>
+        <v>37.513705709523812</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.3">
@@ -3603,12 +3603,12 @@
         <v>20</v>
       </c>
       <c r="F146" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G146" s="3"/>
       <c r="H146">
         <f t="shared" si="8"/>
-        <v>44.754441256666695</v>
+        <v>38.895182419047622</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.3">
@@ -3624,12 +3624,12 @@
         <v>20</v>
       </c>
       <c r="F147" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G147" s="3"/>
       <c r="H147">
         <f t="shared" si="8"/>
-        <v>46.246255965222254</v>
+        <v>40.276659128571431</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.3">
@@ -3645,12 +3645,12 @@
         <v>20</v>
       </c>
       <c r="F148" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G148" s="4"/>
       <c r="H148">
         <f t="shared" si="8"/>
-        <v>47.738070673777813</v>
+        <v>41.658135838095241</v>
       </c>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.3">
@@ -3666,12 +3666,12 @@
         <v>20</v>
       </c>
       <c r="F149" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G149" s="3"/>
       <c r="H149">
         <f t="shared" si="8"/>
-        <v>49.229885382333372</v>
+        <v>43.039612547619051</v>
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.3">
@@ -3687,12 +3687,12 @@
         <v>20</v>
       </c>
       <c r="F150" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G150" s="3"/>
       <c r="H150">
         <f t="shared" si="8"/>
-        <v>50.72170009088893</v>
+        <v>44.42108925714286</v>
       </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.3">
@@ -3708,12 +3708,12 @@
         <v>20</v>
       </c>
       <c r="F151" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G151" s="3"/>
       <c r="H151">
         <f t="shared" si="8"/>
-        <v>52.213514799444489</v>
+        <v>45.80256596666667</v>
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.3">
@@ -3729,12 +3729,12 @@
         <v>20</v>
       </c>
       <c r="F152" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G152" s="3"/>
       <c r="H152">
         <f t="shared" si="8"/>
-        <v>53.705329508000048</v>
+        <v>47.184042676190479</v>
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.3">
@@ -3750,12 +3750,12 @@
         <v>20</v>
       </c>
       <c r="F153" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G153" s="3"/>
       <c r="H153">
         <f t="shared" si="8"/>
-        <v>55.197144216555607</v>
+        <v>48.565519385714289</v>
       </c>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.3">
@@ -3771,12 +3771,12 @@
         <v>20</v>
       </c>
       <c r="F154" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G154" s="3"/>
       <c r="H154">
         <f t="shared" si="8"/>
-        <v>56.688958925111166</v>
+        <v>49.946996095238099</v>
       </c>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.3">
@@ -3792,12 +3792,12 @@
         <v>20</v>
       </c>
       <c r="F155" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G155" s="4"/>
       <c r="H155">
         <f t="shared" si="8"/>
-        <v>58.180773633666725</v>
+        <v>51.328472804761908</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.3">
@@ -3813,12 +3813,12 @@
         <v>20</v>
       </c>
       <c r="F156" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G156" s="3"/>
       <c r="H156">
         <f t="shared" si="8"/>
-        <v>59.672588342222284</v>
+        <v>52.709949514285718</v>
       </c>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.3">
@@ -3834,12 +3834,12 @@
         <v>20</v>
       </c>
       <c r="F157" s="6">
-        <v>1491.8147085555559</v>
+        <v>1381.4767095238096</v>
       </c>
       <c r="G157" s="3"/>
       <c r="H157">
         <f t="shared" si="8"/>
-        <v>61.164403050777842</v>
+        <v>54.091426223809528</v>
       </c>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.3">
@@ -3855,12 +3855,12 @@
         <v>20</v>
       </c>
       <c r="F158" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G158" s="3"/>
       <c r="H158">
         <f t="shared" si="8"/>
-        <v>62.656217759333401</v>
+        <v>55.760026223809525</v>
       </c>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.3">
@@ -3876,12 +3876,12 @@
         <v>20</v>
       </c>
       <c r="F159" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G159" s="3"/>
       <c r="H159">
         <f t="shared" si="8"/>
-        <v>64.148032467888953</v>
+        <v>57.428626223809523</v>
       </c>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.3">
@@ -3897,12 +3897,12 @@
         <v>20</v>
       </c>
       <c r="F160" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G160" s="3"/>
       <c r="H160">
         <f t="shared" si="8"/>
-        <v>65.639847176444505</v>
+        <v>59.097226223809521</v>
       </c>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.3">
@@ -3918,12 +3918,12 @@
         <v>20</v>
       </c>
       <c r="F161" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G161" s="3"/>
       <c r="H161">
         <f t="shared" si="8"/>
-        <v>67.131661885000057</v>
+        <v>60.765826223809519</v>
       </c>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.3">
@@ -3939,12 +3939,12 @@
         <v>20</v>
       </c>
       <c r="F162" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G162" s="4"/>
       <c r="H162">
         <f t="shared" si="8"/>
-        <v>68.623476593555608</v>
+        <v>62.434426223809517</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.3">
@@ -3960,12 +3960,12 @@
         <v>20</v>
       </c>
       <c r="F163" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G163" s="4"/>
       <c r="H163">
         <f t="shared" si="8"/>
-        <v>70.11529130211116</v>
+        <v>64.103026223809522</v>
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.3">
@@ -3981,12 +3981,12 @@
         <v>20</v>
       </c>
       <c r="F164" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G164" s="4"/>
       <c r="H164">
         <f t="shared" si="8"/>
-        <v>71.607106010666712</v>
+        <v>65.77162622380952</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.3">
@@ -4002,12 +4002,12 @@
         <v>20</v>
       </c>
       <c r="F165" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G165" s="4"/>
       <c r="H165">
         <f t="shared" si="8"/>
-        <v>73.098920719222264</v>
+        <v>67.440226223809518</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.3">
@@ -4023,12 +4023,12 @@
         <v>20</v>
       </c>
       <c r="F166" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G166" s="4"/>
       <c r="H166">
         <f t="shared" si="8"/>
-        <v>74.590735427777815</v>
+        <v>69.108826223809515</v>
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.3">
@@ -4044,12 +4044,12 @@
         <v>20</v>
       </c>
       <c r="F167" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G167" s="4"/>
       <c r="H167">
         <f t="shared" si="8"/>
-        <v>76.082550136333367</v>
+        <v>70.777426223809513</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.3">
@@ -4065,12 +4065,12 @@
         <v>20</v>
       </c>
       <c r="F168" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G168" s="4"/>
       <c r="H168">
         <f t="shared" si="8"/>
-        <v>77.574364844888919</v>
+        <v>72.446026223809511</v>
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.3">
@@ -4086,12 +4086,12 @@
         <v>20</v>
       </c>
       <c r="F169" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G169" s="4"/>
       <c r="H169">
         <f t="shared" si="8"/>
-        <v>79.066179553444471</v>
+        <v>74.114626223809509</v>
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.3">
@@ -4107,12 +4107,12 @@
         <v>20</v>
       </c>
       <c r="F170" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G170" s="4"/>
       <c r="H170">
         <f t="shared" si="8"/>
-        <v>80.557994262000022</v>
+        <v>75.783226223809507</v>
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.3">
@@ -4128,12 +4128,12 @@
         <v>20</v>
       </c>
       <c r="F171" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G171" s="4"/>
       <c r="H171">
         <f t="shared" si="8"/>
-        <v>82.049808970555574</v>
+        <v>77.451826223809505</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.3">
@@ -4149,12 +4149,12 @@
         <v>20</v>
       </c>
       <c r="F172" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G172" s="4"/>
       <c r="H172">
         <f t="shared" si="8"/>
-        <v>83.541623679111126</v>
+        <v>79.120426223809503</v>
       </c>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.3">
@@ -4170,12 +4170,12 @@
         <v>20</v>
       </c>
       <c r="F173" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G173" s="4"/>
       <c r="H173">
         <f t="shared" si="8"/>
-        <v>85.033438387666678</v>
+        <v>80.7890262238095</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.3">
@@ -4191,12 +4191,12 @@
         <v>20</v>
       </c>
       <c r="F174" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G174" s="4"/>
       <c r="H174">
         <f t="shared" si="8"/>
-        <v>86.525253096222229</v>
+        <v>82.457626223809498</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.3">
@@ -4212,12 +4212,12 @@
         <v>20</v>
       </c>
       <c r="F175" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G175" s="4"/>
       <c r="H175">
         <f t="shared" si="8"/>
-        <v>88.017067804777781</v>
+        <v>84.126226223809496</v>
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.3">
@@ -4233,12 +4233,12 @@
         <v>20</v>
       </c>
       <c r="F176" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G176" s="4"/>
       <c r="H176">
         <f t="shared" si="8"/>
-        <v>89.508882513333333</v>
+        <v>85.794826223809494</v>
       </c>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.3">
@@ -4254,12 +4254,12 @@
         <v>20</v>
       </c>
       <c r="F177" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G177" s="4"/>
       <c r="H177">
         <f t="shared" si="8"/>
-        <v>91.000697221888885</v>
+        <v>87.463426223809492</v>
       </c>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.3">
@@ -4275,12 +4275,12 @@
         <v>20</v>
       </c>
       <c r="F178" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G178" s="4"/>
       <c r="H178">
         <f t="shared" si="8"/>
-        <v>92.492511930444437</v>
+        <v>89.13202622380949</v>
       </c>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.3">
@@ -4296,12 +4296,12 @@
         <v>20</v>
       </c>
       <c r="F179" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G179" s="4"/>
       <c r="H179">
         <f t="shared" si="8"/>
-        <v>93.984326638999988</v>
+        <v>90.800626223809488</v>
       </c>
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.3">
@@ -4317,12 +4317,12 @@
         <v>20</v>
       </c>
       <c r="F180" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G180" s="4"/>
       <c r="H180">
         <f t="shared" si="8"/>
-        <v>95.47614134755554</v>
+        <v>92.469226223809486</v>
       </c>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.3">
@@ -4338,12 +4338,12 @@
         <v>20</v>
       </c>
       <c r="F181" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G181" s="4"/>
       <c r="H181">
         <f t="shared" si="8"/>
-        <v>96.967956056111092</v>
+        <v>94.137826223809483</v>
       </c>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.3">
@@ -4359,14 +4359,14 @@
         <v>20</v>
       </c>
       <c r="F182" s="6">
-        <v>1491.8147085555559</v>
+        <v>1668.5999999999995</v>
       </c>
       <c r="G182" s="4">
         <v>51.4</v>
       </c>
       <c r="H182">
         <f t="shared" si="8"/>
-        <v>98.459770764666644</v>
+        <v>95.806426223809481</v>
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.3">
@@ -4381,7 +4381,7 @@
         <v>21</v>
       </c>
       <c r="F183" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G183" s="4">
         <v>40.799999999999997</v>
@@ -4400,12 +4400,12 @@
         <v>21</v>
       </c>
       <c r="F184" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G184" s="3"/>
       <c r="H184">
         <f t="shared" ref="H184:H186" si="13">H183+F184/1000</f>
-        <v>1.0317450394444443</v>
+        <v>1.1534659166666668</v>
       </c>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.3">
@@ -4421,12 +4421,12 @@
         <v>21</v>
       </c>
       <c r="F185" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G185" s="3"/>
       <c r="H185">
         <f t="shared" si="13"/>
-        <v>2.0634900788888886</v>
+        <v>2.3069318333333335</v>
       </c>
     </row>
     <row r="186" spans="1:8" x14ac:dyDescent="0.3">
@@ -4442,12 +4442,12 @@
         <v>21</v>
       </c>
       <c r="F186" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G186" s="3"/>
       <c r="H186">
         <f t="shared" si="13"/>
-        <v>3.0952351183333331</v>
+        <v>3.4603977500000003</v>
       </c>
     </row>
     <row r="187" spans="1:8" x14ac:dyDescent="0.3">
@@ -4463,12 +4463,12 @@
         <v>21</v>
       </c>
       <c r="F187" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G187" s="4"/>
       <c r="H187">
         <f t="shared" ref="H187:H249" si="14">H186+F187/1000</f>
-        <v>4.1269801577777772</v>
+        <v>4.613863666666667</v>
       </c>
     </row>
     <row r="188" spans="1:8" x14ac:dyDescent="0.3">
@@ -4484,12 +4484,12 @@
         <v>21</v>
       </c>
       <c r="F188" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G188" s="3"/>
       <c r="H188">
         <f t="shared" si="14"/>
-        <v>5.1587251972222212</v>
+        <v>5.7673295833333338</v>
       </c>
     </row>
     <row r="189" spans="1:8" x14ac:dyDescent="0.3">
@@ -4505,12 +4505,12 @@
         <v>21</v>
       </c>
       <c r="F189" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G189" s="3"/>
       <c r="H189">
         <f t="shared" si="14"/>
-        <v>6.1904702366666653</v>
+        <v>6.9207955000000005</v>
       </c>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.3">
@@ -4526,12 +4526,12 @@
         <v>21</v>
       </c>
       <c r="F190" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G190" s="3"/>
       <c r="H190">
         <f t="shared" si="14"/>
-        <v>7.2222152761111094</v>
+        <v>8.0742614166666673</v>
       </c>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.3">
@@ -4547,12 +4547,12 @@
         <v>21</v>
       </c>
       <c r="F191" s="6">
-        <v>1031.7450394444443</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G191" s="3"/>
       <c r="H191">
         <f t="shared" si="14"/>
-        <v>8.2539603155555543</v>
+        <v>9.2277273333333341</v>
       </c>
     </row>
     <row r="192" spans="1:8" x14ac:dyDescent="0.3">
@@ -4568,12 +4568,12 @@
         <v>21</v>
       </c>
       <c r="F192" s="6">
-        <v>1031.74503944444</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G192" s="3"/>
       <c r="H192">
         <f t="shared" si="14"/>
-        <v>9.2857053549999939</v>
+        <v>10.381193250000001</v>
       </c>
     </row>
     <row r="193" spans="1:8" x14ac:dyDescent="0.3">
@@ -4589,12 +4589,12 @@
         <v>21</v>
       </c>
       <c r="F193" s="6">
-        <v>1031.74503944444</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G193" s="3"/>
       <c r="H193">
         <f t="shared" si="14"/>
-        <v>10.317450394444434</v>
+        <v>11.534659166666668</v>
       </c>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.3">
@@ -4610,12 +4610,12 @@
         <v>21</v>
       </c>
       <c r="F194" s="6">
-        <v>1031.74503944444</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G194" s="4"/>
       <c r="H194">
         <f t="shared" si="14"/>
-        <v>11.349195433888873</v>
+        <v>12.688125083333334</v>
       </c>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.3">
@@ -4631,12 +4631,12 @@
         <v>21</v>
       </c>
       <c r="F195" s="6">
-        <v>1031.74503944444</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G195" s="3"/>
       <c r="H195">
         <f t="shared" si="14"/>
-        <v>12.380940473333313</v>
+        <v>13.841591000000001</v>
       </c>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.3">
@@ -4652,12 +4652,12 @@
         <v>21</v>
       </c>
       <c r="F196" s="6">
-        <v>1031.74503944444</v>
+        <v>1153.4659166666668</v>
       </c>
       <c r="G196" s="3"/>
       <c r="H196">
         <f t="shared" si="14"/>
-        <v>13.412685512777752</v>
+        <v>14.995056916666668</v>
       </c>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.3">
@@ -4673,12 +4673,12 @@
         <v>21</v>
       </c>
       <c r="F197" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G197" s="3"/>
       <c r="H197">
         <f t="shared" si="14"/>
-        <v>14.444430552222192</v>
+        <v>15.910461977777778</v>
       </c>
     </row>
     <row r="198" spans="1:8" x14ac:dyDescent="0.3">
@@ -4694,12 +4694,12 @@
         <v>21</v>
       </c>
       <c r="F198" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G198" s="3"/>
       <c r="H198">
         <f t="shared" si="14"/>
-        <v>15.476175591666632</v>
+        <v>16.825867038888891</v>
       </c>
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.3">
@@ -4715,12 +4715,12 @@
         <v>21</v>
       </c>
       <c r="F199" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G199" s="3"/>
       <c r="H199">
         <f t="shared" si="14"/>
-        <v>16.507920631111073</v>
+        <v>17.741272100000003</v>
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.3">
@@ -4736,12 +4736,12 @@
         <v>21</v>
       </c>
       <c r="F200" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G200" s="3"/>
       <c r="H200">
         <f t="shared" si="14"/>
-        <v>17.539665670555515</v>
+        <v>18.656677161111116</v>
       </c>
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.3">
@@ -4757,12 +4757,12 @@
         <v>21</v>
       </c>
       <c r="F201" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G201" s="4"/>
       <c r="H201">
         <f t="shared" si="14"/>
-        <v>18.571410709999956</v>
+        <v>19.572082222222228</v>
       </c>
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.3">
@@ -4778,12 +4778,12 @@
         <v>21</v>
       </c>
       <c r="F202" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G202" s="3"/>
       <c r="H202">
         <f t="shared" si="14"/>
-        <v>19.603155749444397</v>
+        <v>20.487487283333341</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.3">
@@ -4799,12 +4799,12 @@
         <v>21</v>
       </c>
       <c r="F203" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G203" s="3"/>
       <c r="H203">
         <f t="shared" si="14"/>
-        <v>20.634900788888839</v>
+        <v>21.402892344444453</v>
       </c>
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.3">
@@ -4820,12 +4820,12 @@
         <v>21</v>
       </c>
       <c r="F204" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G204" s="3"/>
       <c r="H204">
         <f t="shared" si="14"/>
-        <v>21.66664582833328</v>
+        <v>22.318297405555565</v>
       </c>
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.3">
@@ -4841,12 +4841,12 @@
         <v>21</v>
       </c>
       <c r="F205" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G205" s="3"/>
       <c r="H205">
         <f t="shared" si="14"/>
-        <v>22.698390867777722</v>
+        <v>23.233702466666678</v>
       </c>
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.3">
@@ -4862,12 +4862,12 @@
         <v>21</v>
       </c>
       <c r="F206" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G206" s="3"/>
       <c r="H206">
         <f t="shared" si="14"/>
-        <v>23.730135907222163</v>
+        <v>24.14910752777779</v>
       </c>
     </row>
     <row r="207" spans="1:8" x14ac:dyDescent="0.3">
@@ -4883,12 +4883,12 @@
         <v>21</v>
       </c>
       <c r="F207" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G207" s="3"/>
       <c r="H207">
         <f t="shared" si="14"/>
-        <v>24.761880946666604</v>
+        <v>25.064512588888903</v>
       </c>
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.3">
@@ -4904,12 +4904,12 @@
         <v>21</v>
       </c>
       <c r="F208" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G208" s="4"/>
       <c r="H208">
         <f t="shared" si="14"/>
-        <v>25.793625986111046</v>
+        <v>25.979917650000015</v>
       </c>
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.3">
@@ -4925,12 +4925,12 @@
         <v>21</v>
       </c>
       <c r="F209" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G209" s="3"/>
       <c r="H209">
         <f t="shared" si="14"/>
-        <v>26.825371025555487</v>
+        <v>26.895322711111127</v>
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.3">
@@ -4946,12 +4946,12 @@
         <v>21</v>
       </c>
       <c r="F210" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G210" s="3"/>
       <c r="H210">
         <f t="shared" si="14"/>
-        <v>27.857116064999929</v>
+        <v>27.81072777222224</v>
       </c>
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.3">
@@ -4967,12 +4967,12 @@
         <v>21</v>
       </c>
       <c r="F211" s="6">
-        <v>1031.74503944444</v>
+        <v>915.40506111111119</v>
       </c>
       <c r="G211" s="3"/>
       <c r="H211">
         <f t="shared" si="14"/>
-        <v>28.88886110444437</v>
+        <v>28.726132833333352</v>
       </c>
     </row>
     <row r="212" spans="1:8" x14ac:dyDescent="0.3">
@@ -4988,12 +4988,12 @@
         <v>21</v>
       </c>
       <c r="F212" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G212" s="3"/>
       <c r="H212">
         <f t="shared" si="14"/>
-        <v>29.920606143888811</v>
+        <v>29.738879837407428</v>
       </c>
     </row>
     <row r="213" spans="1:8" x14ac:dyDescent="0.3">
@@ -5009,12 +5009,12 @@
         <v>21</v>
       </c>
       <c r="F213" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G213" s="3"/>
       <c r="H213">
         <f t="shared" si="14"/>
-        <v>30.952351183333253</v>
+        <v>30.751626841481503</v>
       </c>
     </row>
     <row r="214" spans="1:8" x14ac:dyDescent="0.3">
@@ -5030,12 +5030,12 @@
         <v>21</v>
       </c>
       <c r="F214" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G214" s="3"/>
       <c r="H214">
         <f t="shared" si="14"/>
-        <v>31.984096222777694</v>
+        <v>31.764373845555578</v>
       </c>
     </row>
     <row r="215" spans="1:8" x14ac:dyDescent="0.3">
@@ -5051,12 +5051,12 @@
         <v>21</v>
       </c>
       <c r="F215" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G215" s="4"/>
       <c r="H215">
         <f t="shared" si="14"/>
-        <v>33.015841262222132</v>
+        <v>32.777120849629654</v>
       </c>
     </row>
     <row r="216" spans="1:8" x14ac:dyDescent="0.3">
@@ -5072,12 +5072,12 @@
         <v>21</v>
       </c>
       <c r="F216" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G216" s="3"/>
       <c r="H216">
         <f t="shared" si="14"/>
-        <v>34.04758630166657</v>
+        <v>33.789867853703726</v>
       </c>
     </row>
     <row r="217" spans="1:8" x14ac:dyDescent="0.3">
@@ -5093,12 +5093,12 @@
         <v>21</v>
       </c>
       <c r="F217" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G217" s="3"/>
       <c r="H217">
         <f t="shared" si="14"/>
-        <v>35.079331341111008</v>
+        <v>34.802614857777797</v>
       </c>
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.3">
@@ -5114,12 +5114,12 @@
         <v>21</v>
       </c>
       <c r="F218" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G218" s="3"/>
       <c r="H218">
         <f t="shared" si="14"/>
-        <v>36.111076380555446</v>
+        <v>35.815361861851869</v>
       </c>
     </row>
     <row r="219" spans="1:8" x14ac:dyDescent="0.3">
@@ -5135,12 +5135,12 @@
         <v>21</v>
       </c>
       <c r="F219" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G219" s="3"/>
       <c r="H219">
         <f t="shared" si="14"/>
-        <v>37.142821419999883</v>
+        <v>36.828108865925941</v>
       </c>
     </row>
     <row r="220" spans="1:8" x14ac:dyDescent="0.3">
@@ -5156,12 +5156,12 @@
         <v>21</v>
       </c>
       <c r="F220" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G220" s="3"/>
       <c r="H220">
         <f t="shared" si="14"/>
-        <v>38.174566459444321</v>
+        <v>37.840855870000013</v>
       </c>
     </row>
     <row r="221" spans="1:8" x14ac:dyDescent="0.3">
@@ -5177,12 +5177,12 @@
         <v>21</v>
       </c>
       <c r="F221" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G221" s="3"/>
       <c r="H221">
         <f t="shared" si="14"/>
-        <v>39.206311498888759</v>
+        <v>38.853602874074085</v>
       </c>
     </row>
     <row r="222" spans="1:8" x14ac:dyDescent="0.3">
@@ -5198,12 +5198,12 @@
         <v>21</v>
       </c>
       <c r="F222" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G222" s="4"/>
       <c r="H222">
         <f t="shared" si="14"/>
-        <v>40.238056538333197</v>
+        <v>39.866349878148156</v>
       </c>
     </row>
     <row r="223" spans="1:8" x14ac:dyDescent="0.3">
@@ -5219,12 +5219,12 @@
         <v>21</v>
       </c>
       <c r="F223" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G223" s="3"/>
       <c r="H223">
         <f t="shared" si="14"/>
-        <v>41.269801577777635</v>
+        <v>40.879096882222228</v>
       </c>
     </row>
     <row r="224" spans="1:8" x14ac:dyDescent="0.3">
@@ -5240,12 +5240,12 @@
         <v>21</v>
       </c>
       <c r="F224" s="6">
-        <v>1031.74503944444</v>
+        <v>1012.7470040740742</v>
       </c>
       <c r="G224" s="3"/>
       <c r="H224">
         <f t="shared" si="14"/>
-        <v>42.301546617222073</v>
+        <v>41.8918438862963</v>
       </c>
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.3">
@@ -5261,12 +5261,12 @@
         <v>21</v>
       </c>
       <c r="F225" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="G225" s="3"/>
       <c r="H225">
         <f t="shared" si="14"/>
-        <v>43.333291656666511</v>
+        <v>42.9115438862963</v>
       </c>
     </row>
     <row r="226" spans="1:8" x14ac:dyDescent="0.3">
@@ -5282,12 +5282,12 @@
         <v>21</v>
       </c>
       <c r="F226" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="G226" s="3"/>
       <c r="H226">
         <f t="shared" si="14"/>
-        <v>44.365036696110948</v>
+        <v>43.931243886296301</v>
       </c>
     </row>
     <row r="227" spans="1:8" x14ac:dyDescent="0.3">
@@ -5303,12 +5303,12 @@
         <v>21</v>
       </c>
       <c r="F227" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="G227" s="3"/>
       <c r="H227">
         <f t="shared" si="14"/>
-        <v>45.396781735555386</v>
+        <v>44.950943886296301</v>
       </c>
     </row>
     <row r="228" spans="1:8" x14ac:dyDescent="0.3">
@@ -5324,12 +5324,12 @@
         <v>21</v>
       </c>
       <c r="F228" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="G228" s="3"/>
       <c r="H228">
         <f t="shared" si="14"/>
-        <v>46.428526774999824</v>
+        <v>45.970643886296301</v>
       </c>
     </row>
     <row r="229" spans="1:8" x14ac:dyDescent="0.3">
@@ -5345,12 +5345,12 @@
         <v>21</v>
       </c>
       <c r="F229" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="G229" s="4"/>
       <c r="H229">
         <f t="shared" si="14"/>
-        <v>47.460271814444262</v>
+        <v>46.990343886296301</v>
       </c>
     </row>
     <row r="230" spans="1:8" x14ac:dyDescent="0.3">
@@ -5366,11 +5366,11 @@
         <v>21</v>
       </c>
       <c r="F230" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H230">
         <f t="shared" si="14"/>
-        <v>48.4920168538887</v>
+        <v>48.010043886296302</v>
       </c>
     </row>
     <row r="231" spans="1:8" x14ac:dyDescent="0.3">
@@ -5386,11 +5386,11 @@
         <v>21</v>
       </c>
       <c r="F231" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H231">
         <f t="shared" si="14"/>
-        <v>49.523761893333138</v>
+        <v>49.029743886296302</v>
       </c>
     </row>
     <row r="232" spans="1:8" x14ac:dyDescent="0.3">
@@ -5406,11 +5406,11 @@
         <v>21</v>
       </c>
       <c r="F232" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H232">
         <f t="shared" si="14"/>
-        <v>50.555506932777575</v>
+        <v>50.049443886296302</v>
       </c>
     </row>
     <row r="233" spans="1:8" x14ac:dyDescent="0.3">
@@ -5426,11 +5426,11 @@
         <v>21</v>
       </c>
       <c r="F233" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H233">
         <f t="shared" si="14"/>
-        <v>51.587251972222013</v>
+        <v>51.069143886296303</v>
       </c>
     </row>
     <row r="234" spans="1:8" x14ac:dyDescent="0.3">
@@ -5446,11 +5446,11 @@
         <v>21</v>
       </c>
       <c r="F234" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H234">
         <f t="shared" si="14"/>
-        <v>52.618997011666451</v>
+        <v>52.088843886296303</v>
       </c>
     </row>
     <row r="235" spans="1:8" x14ac:dyDescent="0.3">
@@ -5466,11 +5466,11 @@
         <v>21</v>
       </c>
       <c r="F235" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H235">
         <f t="shared" si="14"/>
-        <v>53.650742051110889</v>
+        <v>53.108543886296303</v>
       </c>
     </row>
     <row r="236" spans="1:8" x14ac:dyDescent="0.3">
@@ -5486,11 +5486,11 @@
         <v>21</v>
       </c>
       <c r="F236" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H236">
         <f t="shared" si="14"/>
-        <v>54.682487090555327</v>
+        <v>54.128243886296303</v>
       </c>
     </row>
     <row r="237" spans="1:8" x14ac:dyDescent="0.3">
@@ -5506,11 +5506,11 @@
         <v>21</v>
       </c>
       <c r="F237" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H237">
         <f t="shared" si="14"/>
-        <v>55.714232129999765</v>
+        <v>55.147943886296304</v>
       </c>
     </row>
     <row r="238" spans="1:8" x14ac:dyDescent="0.3">
@@ -5526,11 +5526,11 @@
         <v>21</v>
       </c>
       <c r="F238" s="6">
-        <v>1031.74503944444</v>
+        <v>1019.7000000000003</v>
       </c>
       <c r="H238">
         <f t="shared" si="14"/>
-        <v>56.745977169444203</v>
+        <v>56.167643886296304</v>
       </c>
     </row>
     <row r="239" spans="1:8" x14ac:dyDescent="0.3">
@@ -5546,11 +5546,11 @@
         <v>21</v>
       </c>
       <c r="F239" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H239">
         <f t="shared" si="14"/>
-        <v>57.77772220888864</v>
+        <v>57.27110161356903</v>
       </c>
     </row>
     <row r="240" spans="1:8" x14ac:dyDescent="0.3">
@@ -5566,11 +5566,11 @@
         <v>21</v>
       </c>
       <c r="F240" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H240">
         <f t="shared" si="14"/>
-        <v>58.809467248333078</v>
+        <v>58.374559340841756</v>
       </c>
     </row>
     <row r="241" spans="1:8" x14ac:dyDescent="0.3">
@@ -5586,11 +5586,11 @@
         <v>21</v>
       </c>
       <c r="F241" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H241">
         <f t="shared" si="14"/>
-        <v>59.841212287777516</v>
+        <v>59.478017068114482</v>
       </c>
     </row>
     <row r="242" spans="1:8" x14ac:dyDescent="0.3">
@@ -5606,11 +5606,11 @@
         <v>21</v>
       </c>
       <c r="F242" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H242">
         <f t="shared" si="14"/>
-        <v>60.872957327221954</v>
+        <v>60.581474795387209</v>
       </c>
     </row>
     <row r="243" spans="1:8" x14ac:dyDescent="0.3">
@@ -5626,11 +5626,11 @@
         <v>21</v>
       </c>
       <c r="F243" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H243">
         <f t="shared" si="14"/>
-        <v>61.904702366666392</v>
+        <v>61.684932522659935</v>
       </c>
     </row>
     <row r="244" spans="1:8" x14ac:dyDescent="0.3">
@@ -5646,11 +5646,11 @@
         <v>21</v>
       </c>
       <c r="F244" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H244">
         <f t="shared" si="14"/>
-        <v>62.93644740611083</v>
+        <v>62.788390249932661</v>
       </c>
     </row>
     <row r="245" spans="1:8" x14ac:dyDescent="0.3">
@@ -5666,11 +5666,11 @@
         <v>21</v>
       </c>
       <c r="F245" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H245">
         <f t="shared" si="14"/>
-        <v>63.968192445555268</v>
+        <v>63.891847977205387</v>
       </c>
     </row>
     <row r="246" spans="1:8" x14ac:dyDescent="0.3">
@@ -5686,11 +5686,11 @@
         <v>21</v>
       </c>
       <c r="F246" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H246">
         <f t="shared" si="14"/>
-        <v>64.999937484999705</v>
+        <v>64.995305704478113</v>
       </c>
     </row>
     <row r="247" spans="1:8" x14ac:dyDescent="0.3">
@@ -5706,11 +5706,11 @@
         <v>21</v>
       </c>
       <c r="F247" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H247">
         <f t="shared" si="14"/>
-        <v>66.03168252444415</v>
+        <v>66.098763431750839</v>
       </c>
     </row>
     <row r="248" spans="1:8" x14ac:dyDescent="0.3">
@@ -5726,11 +5726,11 @@
         <v>21</v>
       </c>
       <c r="F248" s="6">
-        <v>1031.74503944444</v>
+        <v>1103.4577272727288</v>
       </c>
       <c r="H248">
         <f t="shared" si="14"/>
-        <v>67.063427563888595</v>
+        <v>67.202221159023566</v>
       </c>
     </row>
     <row r="249" spans="1:8" x14ac:dyDescent="0.3">
@@ -5746,14 +5746,14 @@
         <v>21</v>
       </c>
       <c r="F249" s="6">
-        <v>1031.74503944444</v>
-      </c>
-      <c r="G249">
+        <v>1103.4577272727288</v>
+      </c>
+      <c r="G249" s="5">
         <v>45</v>
       </c>
       <c r="H249">
         <f t="shared" si="14"/>
-        <v>68.09517260333304</v>
+        <v>68.305678886296292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>